<commit_message>
fixed motor module select output excel v1
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -17,13 +17,23 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Courier"/>
+      <color rgb="008A3F2F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Courier"/>
+      <color rgb="002F468A"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +56,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
@@ -413,99 +429,107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" max="1" min="1" width="25"/>
+    <col customWidth="1" max="2" min="2" width="25"/>
+    <col customWidth="1" max="3" min="3" width="25"/>
+    <col customWidth="1" max="4" min="4" width="25"/>
+    <col customWidth="1" max="5" min="5" width="25"/>
+    <col customWidth="1" max="6" min="6" width="25"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 1</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 2</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 3</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 4</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 5</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>關節型號 axis 6</t>
+    <row customHeight="1" ht="40" r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 1</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 2</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 3</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 4</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 5</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 6</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>static</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>static analysis result</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="A3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>dynamic analysis result</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="A6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>static</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>static analysis input data</t>
         </is>
       </c>
     </row>
@@ -546,9 +570,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>dynamic analysis input data</t>
         </is>
       </c>
     </row>
@@ -692,12 +716,183 @@
         <v>0</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>The selected joint module model</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>model number</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>rated_torque</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>rated_speed</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>max_torque</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>max_output_speed</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>diameter</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0</v>
+      </c>
+      <c r="B22" t="n">
+        <v>16</v>
+      </c>
+      <c r="C22" t="n">
+        <v>35</v>
+      </c>
+      <c r="D22" t="n">
+        <v>32</v>
+      </c>
+      <c r="E22" t="n">
+        <v>44</v>
+      </c>
+      <c r="F22" t="n">
+        <v>80</v>
+      </c>
+      <c r="G22" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>123</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="n">
+        <v>38</v>
+      </c>
+      <c r="C23" t="n">
+        <v>25</v>
+      </c>
+      <c r="D23" t="n">
+        <v>66</v>
+      </c>
+      <c r="E23" t="n">
+        <v>31</v>
+      </c>
+      <c r="F23" t="n">
+        <v>90</v>
+      </c>
+      <c r="G23" t="n">
+        <v>105</v>
+      </c>
+      <c r="H23" t="n">
+        <v>125</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" t="n">
+        <v>60</v>
+      </c>
+      <c r="C24" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>120</v>
+      </c>
+      <c r="E24" t="n">
+        <v>42</v>
+      </c>
+      <c r="F24" t="n">
+        <v>102</v>
+      </c>
+      <c r="G24" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>141</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" t="n">
+        <v>114</v>
+      </c>
+      <c r="C25" t="n">
+        <v>15</v>
+      </c>
+      <c r="D25" t="n">
+        <v>198</v>
+      </c>
+      <c r="E25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F25" t="n">
+        <v>130</v>
+      </c>
+      <c r="G25" t="n">
+        <v>145</v>
+      </c>
+      <c r="H25" t="n">
+        <v>130</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A20:I20"/>
   </mergeCells>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>

<commit_message>
arm workspace plane test ok
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -511,10 +511,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -566,7 +566,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +600,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="15">
@@ -646,22 +646,22 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -698,22 +698,22 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
TODO: DQN robot design environment
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -511,10 +511,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -566,7 +566,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +600,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -646,22 +646,22 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -698,22 +698,22 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
add can input axis length information
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -484,10 +484,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>0</v>
@@ -508,13 +508,13 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -566,7 +566,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +600,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="15">
@@ -646,22 +646,22 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
     </row>
     <row r="17">
@@ -698,22 +698,22 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>2.359999895095825</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>3.670000076293945</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
interface add joint 7
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -508,18 +508,16 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>fail</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
@@ -559,7 +557,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -568,7 +566,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -602,7 +600,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -611,7 +609,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -648,22 +646,22 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="B16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -700,22 +698,22 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="B18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>3.150000095367432</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
dynamics 7dof single test ok & scan plot error
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -438,6 +438,7 @@
     <col customWidth="1" max="4" min="4" width="25"/>
     <col customWidth="1" max="5" min="5" width="25"/>
     <col customWidth="1" max="6" min="6" width="25"/>
+    <col customWidth="1" max="7" min="7" width="25"/>
   </cols>
   <sheetData>
     <row customHeight="1" ht="40" r="1">
@@ -471,6 +472,11 @@
           <t>model number of axis 6</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>model number of axis 7</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -484,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>0</v>
@@ -496,6 +502,9 @@
         <v>0</v>
       </c>
       <c r="F3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -511,18 +520,21 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -557,7 +569,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -566,7 +578,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +612,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -609,7 +621,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.03999999910593033</v>
       </c>
     </row>
     <row r="15">
@@ -643,25 +655,30 @@
           <t>velocity of axis 6</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>velocity of axis 7</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
     </row>
     <row r="17">
@@ -695,25 +712,30 @@
           <t>acceralation of axis 6</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>acceralation of axis 7</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1.570000052452087</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
add select sturcture function
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/CJM_select.xlsx
+++ b/dynamics/src/dynamics/xlsx/CJM_select.xlsx
@@ -517,10 +517,10 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>1</v>
@@ -532,7 +532,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>0</v>
@@ -578,7 +578,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -621,7 +621,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03999999910593033</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -663,22 +663,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="B16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="C16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="D16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="E16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="F16" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3.036872863769531</v>
       </c>
     </row>
     <row r="17">
@@ -720,22 +723,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="B18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="C18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="D18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="E18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
       </c>
       <c r="F18" t="n">
-        <v>1.570000052452087</v>
+        <v>3.036872863769531</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3.036872863769531</v>
       </c>
     </row>
     <row r="20">

</xml_diff>